<commit_message>
Punto 4.5: informe de revisión de los itinerarios formativos e itinerarios corregidos
Matriz de cumplimiento de la guía de llenado (23 controles) para las 43
asignaturas, resumen y detalle de observaciones por asignatura, nombres y
diferencias frente a la malla, y correcciones ortográficas aplicadas con
control de cambios en copias de los 39 itinerarios en Word.
Checklist actualizado (filas 4.5-a a 4.5-i).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Li7yxA95TVg4oPXuqG5DZe
</commit_message>
<xml_diff>
--- a/rediseno_2026/Checklist de entregas - Rediseño Curricular 2026 actualizado.xlsx
+++ b/rediseno_2026/Checklist de entregas - Rediseño Curricular 2026 actualizado.xlsx
@@ -3427,21 +3427,31 @@
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="n"/>
-      <c r="G60" s="6" t="n"/>
+          <t>Entregado</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I60" s="10" t="n"/>
+          <t>Revisado</t>
+        </is>
+      </c>
+      <c r="I60" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observado. 6 itinerarios (CPA-101, 201, 202, 203, 301, 302). Estado: 5 ajustes menores y CPA-301 requiere ajustes. Sin cambios de nombre. Horas llenadas en los 6; CPA-301 sin columna «En clase». El informe de la subcomisión declara cambios en CPA-201 que el itinerario solo refleja en parte. Revisado en «4.5 Informe de revisión de los itinerarios formativos.docx» (matriz de cumplimiento de la guía, resumen y detalle por asignatura). Correcciones ortográficas y de forma con control de cambios en la carpeta «4.5 Itinerarios corregidos». </t>
+        </is>
+      </c>
       <c r="J60" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K60" s="10" t="n"/>
+      <c r="K60" s="24" t="n"/>
     </row>
     <row r="61" ht="26.4" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
@@ -3466,21 +3476,31 @@
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="n"/>
-      <c r="G61" s="6" t="n"/>
+          <t>Entregado</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I61" s="10" t="n"/>
+          <t>Revisado</t>
+        </is>
+      </c>
+      <c r="I61" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observado. 7 itinerarios (CPA-303, 304, 401 a 405). Estado: CPA-303 y CPA-404 requieren reformulación parcial; CPA-402 y CPA-403 requieren ajustes; el resto, ajustes menores. Cambios de nombre: CPA-304 («Presupuesto y Contabilidad Gubernamental») y sigla CPA-406 dentro de CPA-405. CPA-404 entregado con 992 cambios controlados sin resolver. Revisado en «4.5 Informe de revisión de los itinerarios formativos.docx» (matriz de cumplimiento de la guía, resumen y detalle por asignatura). Correcciones ortográficas y de forma con control de cambios en la carpeta «4.5 Itinerarios corregidos». </t>
+        </is>
+      </c>
       <c r="J61" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K61" s="10" t="n"/>
+      <c r="K61" s="24" t="n"/>
     </row>
     <row r="62" ht="39.6" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
@@ -3505,21 +3525,31 @@
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="n"/>
-      <c r="G62" s="6" t="n"/>
+          <t>Entregado</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I62" s="10" t="n"/>
+          <t>Revisado</t>
+        </is>
+      </c>
+      <c r="I62" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observado. 11 itinerarios (CPA-406 a 408, 501 a 504, 506 a 509). Estado: CPA-407 requiere reformulación parcial; CPA-408, 502, 504, 506, 507 y 508 requieren ajustes. Cambios de nombre sin justificar: CPA-408, 506, 507 y 508. CPA-504 tiene pegado en la bibliografía un mensaje de un asistente de IA. CPA-507 está todo en fuente Inter. Revisado en «4.5 Informe de revisión de los itinerarios formativos.docx» (matriz de cumplimiento de la guía, resumen y detalle por asignatura). Correcciones ortográficas y de forma con control de cambios en la carpeta «4.5 Itinerarios corregidos». </t>
+        </is>
+      </c>
       <c r="J62" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K62" s="10" t="n"/>
+      <c r="K62" s="24" t="n"/>
     </row>
     <row r="63" ht="26.4" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
@@ -3544,21 +3574,31 @@
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="n"/>
-      <c r="G63" s="6" t="n"/>
+          <t>Entregado</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I63" s="10" t="n"/>
+          <t>Revisado</t>
+        </is>
+      </c>
+      <c r="I63" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observado. 3 itinerarios (CPA-102, 305, 505). Estado: CPA-305 requiere reformulación parcial (no desarrolla ERP ni análisis de datos), CPA-102 requiere ajustes, CPA-505 ajustes menores. Cambios de nombre: CPA-102 y CPA-305. Créditos llenados en los 3. Sin informe de subcomisión. Revisado en «4.5 Informe de revisión de los itinerarios formativos.docx» (matriz de cumplimiento de la guía, resumen y detalle por asignatura). Correcciones ortográficas y de forma con control de cambios en la carpeta «4.5 Itinerarios corregidos». </t>
+        </is>
+      </c>
       <c r="J63" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K63" s="10" t="n"/>
+      <c r="K63" s="24" t="n"/>
     </row>
     <row r="64" ht="26.4" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
@@ -3583,21 +3623,31 @@
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F64" s="9" t="n"/>
-      <c r="G64" s="6" t="n"/>
+          <t>Entregado</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I64" s="10" t="n"/>
+          <t>Revisado</t>
+        </is>
+      </c>
+      <c r="I64" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observado. 3 itinerarios entregados en PDF, no en Word; deben entregarse en Word editable. Estado: ADM-201 requiere reformulación parcial, ADM-301 requiere ajustes, ADM-101 ajustes menores. Correcciones de ADM-201 listadas en el Anexo A del informe. Sin informe de subcomisión. Revisado en «4.5 Informe de revisión de los itinerarios formativos.docx» (matriz de cumplimiento de la guía, resumen y detalle por asignatura). Correcciones ortográficas y de forma con control de cambios en la carpeta «4.5 Itinerarios corregidos». </t>
+        </is>
+      </c>
       <c r="J64" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K64" s="10" t="n"/>
+      <c r="K64" s="24" t="n"/>
     </row>
     <row r="65" ht="39.6" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
@@ -3622,21 +3672,31 @@
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="n"/>
-      <c r="G65" s="6" t="n"/>
+          <t>Entregado</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I65" s="10" t="n"/>
+          <t>Revisado</t>
+        </is>
+      </c>
+      <c r="I65" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observado. 3 itinerarios (DER-101, 102, 201). Estado: DER-201 requiere ajustes; el resto, ajustes menores. Sin cambios de nombre. Sin informe de subcomisión. Revisado en «4.5 Informe de revisión de los itinerarios formativos.docx» (matriz de cumplimiento de la guía, resumen y detalle por asignatura). Correcciones ortográficas y de forma con control de cambios en la carpeta «4.5 Itinerarios corregidos». </t>
+        </is>
+      </c>
       <c r="J65" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K65" s="10" t="n"/>
+      <c r="K65" s="24" t="n"/>
     </row>
     <row r="66" ht="26.4" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
@@ -3661,21 +3721,31 @@
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F66" s="9" t="n"/>
-      <c r="G66" s="6" t="n"/>
+          <t>Entregado</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I66" s="10" t="n"/>
+          <t>Revisado</t>
+        </is>
+      </c>
+      <c r="I66" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observado. 3 itinerarios (ECO-101, 201, 301). Estado: ECO-301 requiere ajustes; el resto, ajustes menores. Sin cambios de nombre. Los cambios que declara el informe de la subcomisión quedaron aplicados solo en parte. Revisado en «4.5 Informe de revisión de los itinerarios formativos.docx» (matriz de cumplimiento de la guía, resumen y detalle por asignatura). Correcciones ortográficas y de forma con control de cambios en la carpeta «4.5 Itinerarios corregidos». </t>
+        </is>
+      </c>
       <c r="J66" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K66" s="10" t="n"/>
+      <c r="K66" s="24" t="n"/>
     </row>
     <row r="67" ht="26.4" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
@@ -3700,21 +3770,31 @@
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F67" s="9" t="n"/>
-      <c r="G67" s="6" t="n"/>
+          <t>Entregado</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I67" s="10" t="n"/>
+          <t>Revisado</t>
+        </is>
+      </c>
+      <c r="I67" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observado. 2 itinerarios (CPA-204, 510). Estado: CPA-510 requiere ajustes (sigla HTC, rótulo «Clases», sin trabajo dirigido, diplomado ni PETAENG); CPA-204, ajustes menores y único que dejó las horas en blanco. Sin informe de subcomisión. Revisado en «4.5 Informe de revisión de los itinerarios formativos.docx» (matriz de cumplimiento de la guía, resumen y detalle por asignatura). Correcciones ortográficas y de forma con control de cambios en la carpeta «4.5 Itinerarios corregidos». </t>
+        </is>
+      </c>
       <c r="J67" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K67" s="10" t="n"/>
+      <c r="K67" s="24" t="n"/>
     </row>
     <row r="68" ht="26.4" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
@@ -3739,21 +3819,31 @@
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="n"/>
-      <c r="G68" s="6" t="n"/>
+          <t>Entregado</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I68" s="10" t="n"/>
+          <t>Revisado</t>
+        </is>
+      </c>
+      <c r="I68" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observado. 5 itinerarios (MAT-101, 102, 201, 301, 401). Estado: MAT-201 y MAT-301 requieren reformulación parcial, MAT-401 requiere ajustes, MAT-101 y MAT-102 ajustes menores. Cambio de nombre: MAT-201 («Álgebra y Programación Lineales»). Sin informe de subcomisión. Revisado en «4.5 Informe de revisión de los itinerarios formativos.docx» (matriz de cumplimiento de la guía, resumen y detalle por asignatura). Correcciones ortográficas y de forma con control de cambios en la carpeta «4.5 Itinerarios corregidos». </t>
+        </is>
+      </c>
       <c r="J68" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K68" s="10" t="n"/>
+      <c r="K68" s="24" t="n"/>
     </row>
     <row r="69" ht="25.2" customHeight="1">
       <c r="A69" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Corrige puntos 1, 2, 4.3, 5 y 13 con documentos pilares
Alinea el punto 5 al Reglamento del Régimen Académico Estudiantil del
Sistema de la Universidad Boliviana (admisión, derechos y obligaciones,
régimen académico, evaluación y modalidades de graduación), incorpora el
Técnico Universitario Medio según la Resolución HCU 426/2024 y cita el
organigrama y los reglamentos internos aprobados por la Resolución HCU
139/2013. Deja como observación para la comisión el examen de grado
técnico superior y el número de asignaturas del Técnico Universitario Medio.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Li7yxA95TVg4oPXuqG5DZe
</commit_message>
<xml_diff>
--- a/rediseno_2026/Checklist de entregas - Rediseño Curricular 2026 actualizado.xlsx
+++ b/rediseno_2026/Checklist de entregas - Rediseño Curricular 2026 actualizado.xlsx
@@ -1062,7 +1062,8 @@
         <is>
           <t>Fuentes: Plan 2027 (Res. HCU 290/2016) y Plan 2024 (3.17.7: Técnico Medio en segundo año y Art. 4 del Reglamento General de Títulos y Grados). CONFIRMAR si el Plan 2027 mantiene el Técnico Medio (Auxiliar en Contabilidad General); el Plan 2027 no lo menciona. Denominación: el Plan 2024 dice "Técnico Superior" y la Res. HCU 290/2016 dice "Técnico Universitario Superior"; se usó la de la resolución. El texto del Plan 2024 sobre el examen de grado técnico superior (3.17.6) corresponde al punto 5.4 y se reserva para ese punto. Errores en el Plan 2027: "Grado (s) académicos intermedios (s)" y espacios dentro de los paréntesis.
 CORRECCIÓN (diagnóstico 2026): se quitó la frase "El Plan de Estudios 2024 reconoce...", porque el plan vigente es el 2013. El Técnico Medio se mantiene sin atribuirlo a un plan y sigue PENDIENTE de confirmación.
-CONFIRMADO por la fuente terciaria (propuesta de plan de estudios, puntos de grados intermedios): mantiene el Técnico Medio (Auxiliar en Contabilidad General) al concluir el segundo año. Esa fuente usa "Técnico Superior en Contabilidad General"; se mantiene "Técnico Universitario Superior" por la Res. HCU 290/2016. Unificar.</t>
+CONFIRMADO por la fuente terciaria (propuesta de plan de estudios, puntos de grados intermedios): mantiene el Técnico Medio (Auxiliar en Contabilidad General) al concluir el segundo año. Esa fuente usa "Técnico Superior en Contabilidad General"; se mantiene "Técnico Universitario Superior" por la Res. HCU 290/2016. Unificar.
+Actualizado el 14/10/2026 con los documentos pilares: Técnico Universitario Medio según HCU 426/2024 (requisito de dos años y graduación directa).</t>
         </is>
       </c>
       <c r="J11" s="6" t="n">
@@ -1210,7 +1211,8 @@
       </c>
       <c r="I14" s="24" t="inlineStr">
         <is>
-          <t>Fuentes: Plan 2027 y Res. HCU 290/2016. Error en el Plan 2027: "Diploma ( s) académico (s) intermedio". Error en el Plan 2024: 1.9 vacío.</t>
+          <t>Fuentes: Plan 2027 y Res. HCU 290/2016. Error en el Plan 2027: "Diploma ( s) académico (s) intermedio". Error en el Plan 2024: 1.9 vacío.
+Actualizado el 14/10/2026 con los documentos pilares: se añade el diploma de Técnico Universitario Medio (HCU 426/2024).</t>
         </is>
       </c>
       <c r="J14" s="6" t="n">
@@ -1308,7 +1310,8 @@
       </c>
       <c r="I16" s="24" t="inlineStr">
         <is>
-          <t>Fuentes: Plan 2027 y Res. HCU 290/2016. Error en el Plan 2027: "Título (s) profesional (s) intermedios". Error en el Plan 2024: 1.11 vacío.</t>
+          <t>Fuentes: Plan 2027 y Res. HCU 290/2016. Error en el Plan 2027: "Título (s) profesional (s) intermedios". Error en el Plan 2024: 1.11 vacío.
+Actualizado el 14/10/2026 con los documentos pilares: se añade el título profesional de Técnico Universitario Medio (HCU 426/2024).</t>
         </is>
       </c>
       <c r="J16" s="6" t="n">
@@ -1753,7 +1756,8 @@
       <c r="I25" s="24" t="inlineStr">
         <is>
           <t>Fuentes: organigrama (imagen) y descripción del documento de la comisión, igual al Plan 2024, y 2.6.1 Plantel administrativo del diagnóstico. Redacción ajustada y sin repeticiones. ERRORES EN LA IMAGEN DEL ORGANIGRAMA (no se pueden corregir en el Word, hay que rehacer la imagen): "KARDIXTA" por "KARDEXISTA", "TRANCRIPTOR" por "TRANSCRIPTOR"; dice "JEFATURA DE CARRERA" mientras el texto dice "Dirección de Carrera"; muestra la Unidad de Postgrado al mismo nivel que el Instituto, mientras el texto dice que depende del Instituto. Incoherencia: el texto del Plan 2024 sobre la Jefatura de Dirección hablaba de "dos secretarias, un profesional contable...", que no coincide con las tablas de personal; se redactó sin cantidades. En las tablas: "Kardixtas I" corregido a "Kardexista I", "Centro de Computo" a "Cómputo", "(item)" a "ítem", y se unificaron las filas repetidas de porteros y becarios. Nombre del Instituto unificado según la Res. HCU 457/2004.
-CORRECCIÓN POSTERIOR: la sigla PETAEG del diagnóstico se unificó a PETAENG (Plan Excepcional de Titulación para Antiguos Estudiantes No Graduados), como en la comisión y el Plan 2024.</t>
+CORRECCIÓN POSTERIOR: la sigla PETAEG del diagnóstico se unificó a PETAENG (Plan Excepcional de Titulación para Antiguos Estudiantes No Graduados), como en la comisión y el Plan 2024.
+Actualizado el 14/10/2026 con los documentos pilares: se cita el organigrama aprobado por HCU 139/2013 y sus diferencias con la estructura actual.</t>
         </is>
       </c>
       <c r="J25" s="6" t="n">
@@ -4127,7 +4131,8 @@
       </c>
       <c r="I74" s="24" t="inlineStr">
         <is>
-          <t>Fuentes: fuente terciaria (5.2.1: tres modalidades con detalle de la Admisión Especial) y comisión (diagnóstico y propuestas 1.1 a 1.3, resumidas en 5.2.1 y 5.2.2). ERROR de la comisión: llama a la PSA "Examen de Suficiencia Académica"; se unificó como Prueba de Suficiencia Académica, igual que en la malla (4.4.3) y en el punto 3. Además, la comisión describe la Admisión Especial como "traspasos de carrera", lo que no coincide con la fuente terciaria ni con la normativa; se usó la lista de la fuente terciaria. Dato agregado: 26,62 % de matrícula no activada (diagnóstico).</t>
+          <t>Fuentes: fuente terciaria (5.2.1: tres modalidades con detalle de la Admisión Especial) y comisión (diagnóstico y propuestas 1.1 a 1.3, resumidas en 5.2.1 y 5.2.2). ERROR de la comisión: llama a la PSA "Examen de Suficiencia Académica"; se unificó como Prueba de Suficiencia Académica, igual que en la malla (4.4.3) y en el punto 3. Además, la comisión describe la Admisión Especial como "traspasos de carrera", lo que no coincide con la fuente terciaria ni con la normativa; se usó la lista de la fuente terciaria. Dato agregado: 26,62 % de matrícula no activada (diagnóstico).
+Actualizado el 14/10/2026 con los documentos pilares: modalidades de admisión alineadas al Reglamento del Régimen Académico Estudiantil (Arts. 4 a 13).</t>
         </is>
       </c>
       <c r="J74" s="6" t="n">
@@ -4176,7 +4181,8 @@
       </c>
       <c r="I75" s="24" t="inlineStr">
         <is>
-          <t>Fuentes: fuente terciaria (5.3.1: régimen, cursos de temporada y mesas de examen), comisión (5.3: diagnóstico y propuestas 2.1 a 2.4) y Plan 2024. FALTABA en todas las fuentes el contenido sobre licencias, suspensiones, reincorporación y abandono que pide el índice; se redactó con el Art. 16 del Reglamento del Régimen Estudiantil (en verde) y reglas generales, sin plazos. PENDIENTE: plazos máximos de suspensión y reincorporación según el reglamento de la UMSA. DECISIONES POR CONFIRMAR: (1) nota previa para recuperar una troncal en verano: Plan 2024 = 20, fuente terciaria = 30, comisión propone eliminarla con tutoría obligatoria; se adoptó la propuesta de la comisión; (2) la comisión habla de un límite de "160 horas" y de "80 horas" para troncales en verano; la norma vigente (Plan 2024) y la fuente terciaria dicen 80 horas, que es lo que se usó; (3) la comisión propone ampliar las mesas de examen a materias prácticas, pero la Res. HCU 352/2021 las limita a materias teóricas; no se incluyó y solo se dejaron los seminarios previos.</t>
+          <t>Fuentes: fuente terciaria (5.3.1: régimen, cursos de temporada y mesas de examen), comisión (5.3: diagnóstico y propuestas 2.1 a 2.4) y Plan 2024. FALTABA en todas las fuentes el contenido sobre licencias, suspensiones, reincorporación y abandono que pide el índice; se redactó con el Art. 16 del Reglamento del Régimen Estudiantil (en verde) y reglas generales, sin plazos. PENDIENTE: plazos máximos de suspensión y reincorporación según el reglamento de la UMSA. DECISIONES POR CONFIRMAR: (1) nota previa para recuperar una troncal en verano: Plan 2024 = 20, fuente terciaria = 30, comisión propone eliminarla con tutoría obligatoria; se adoptó la propuesta de la comisión; (2) la comisión habla de un límite de "160 horas" y de "80 horas" para troncales en verano; la norma vigente (Plan 2024) y la fuente terciaria dicen 80 horas, que es lo que se usó; (3) la comisión propone ampliar las mesas de examen a materias prácticas, pero la Res. HCU 352/2021 las limita a materias teóricas; no se incluyó y solo se dejaron los seminarios previos.
+Actualizado el 14/10/2026 con los documentos pilares: derechos y obligaciones, régimen académico (Arts. 16 a 23), plan global, revisión de calificaciones.</t>
         </is>
       </c>
       <c r="J75" s="6" t="n">
@@ -4229,7 +4235,8 @@
       </c>
       <c r="I76" s="24" t="inlineStr">
         <is>
-          <t>Fuentes: fuente terciaria (5.4: grados y siete modalidades, base de la propuesta) y comisión (5.4: requisitos y plazos actuales, problemas y propuestas 3.1 a 3.4). DECISIONES Y COHERENCIA POR CONFIRMAR: (1) diplomado como modalidad: 800 h (20 créditos, que da 40 h por crédito, distinto de las 30 h del sistema de créditos) en la fuente terciaria y 400 h en el Plan de Desarrollo; se redactó sin cifra ("según la normativa de postgrado"); (2) examen de grado: la comisión dice 4 convocatorias anuales y sorteo de bolos 1 hora antes; la fuente terciaria dice al menos 3 convocatorias y 24 horas; se usaron 4 convocatorias y 24 horas; (3) proyecto de grado: 40/30/30 (comisión, vigente) frente a 45/30/25 (fuente terciaria); se usó la fuente terciaria; (4) trabajo dirigido: se mantiene 85/15 según la Res. HCU 330/2022; la comisión propone reequilibrarlo sin dar cifras; (5) excelencia: se usaron los 75 puntos de la comisión. SIGLA: el diagnóstico decía PETAEG y la comisión y el Plan 2024 PETAENG; se unificó PETAENG (también en el punto 2). Asignatura del examen técnico: "Presupuesto y Contabilidad Gubernamental" se actualizó al nombre de la malla, "Contabilidad y Presupuestos Gubernamental". La fuente terciaria titula al técnico "Técnico Superior en Contabilidad General"; se usó "Técnico Universitario Superior" (Res. HCU 290/2016).</t>
+          <t>Fuentes: fuente terciaria (5.4: grados y siete modalidades, base de la propuesta) y comisión (5.4: requisitos y plazos actuales, problemas y propuestas 3.1 a 3.4). DECISIONES Y COHERENCIA POR CONFIRMAR: (1) diplomado como modalidad: 800 h (20 créditos, que da 40 h por crédito, distinto de las 30 h del sistema de créditos) en la fuente terciaria y 400 h en el Plan de Desarrollo; se redactó sin cifra ("según la normativa de postgrado"); (2) examen de grado: la comisión dice 4 convocatorias anuales y sorteo de bolos 1 hora antes; la fuente terciaria dice al menos 3 convocatorias y 24 horas; se usaron 4 convocatorias y 24 horas; (3) proyecto de grado: 40/30/30 (comisión, vigente) frente a 45/30/25 (fuente terciaria); se usó la fuente terciaria; (4) trabajo dirigido: se mantiene 85/15 según la Res. HCU 330/2022; la comisión propone reequilibrarlo sin dar cifras; (5) excelencia: se usaron los 75 puntos de la comisión. SIGLA: el diagnóstico decía PETAEG y la comisión y el Plan 2024 PETAENG; se unificó PETAENG (también en el punto 2). Asignatura del examen técnico: "Presupuesto y Contabilidad Gubernamental" se actualizó al nombre de la malla, "Contabilidad y Presupuestos Gubernamental". La fuente terciaria titula al técnico "Técnico Superior en Contabilidad General"; se usó "Técnico Universitario Superior" (Res. HCU 290/2016).
+Actualizado el 14/10/2026 con los documentos pilares: Técnico Universitario Medio, correspondencia de modalidades con el Art. 66 y observaciones para la comisión sobre el examen de grado técnico superior y las 16 asignaturas del TUM.</t>
         </is>
       </c>
       <c r="J76" s="6" t="n">
@@ -6202,7 +6209,8 @@
       <c r="I116" s="24" t="inlineStr">
         <is>
           <t>Fuentes: comisión y Plan 2024 (lista de reglamentos, cursos de temporada, mesas de examen y Reglamento de Modalidades de Graduación de 79 artículos) y punto 5. Se agregaron un cuadro de normativa aplicable y un cuadro de reglamentos internos a actualizar o elaborar (prácticas, interacción social, tutoría, evaluación curricular, laboratorios). El reglamento de graduación se reescribió en 46 artículos. CAMBIOS FRENTE A LA COMISIÓN, PARA COHERENCIA CON EL PUNTO 5: (1) proyecto de grado 45/30/25 (comisión 40/30/30); (2) sorteo de bolos con 24 horas de anticipación (comisión: una hora antes); (3) tres reprobaciones de un ciclo ya no inhabilitan de forma definitiva (diplomado o créditos complementarios); (4) recuperación en curso de temporada sin el umbral de 20 puntos, con tutoría obligatoria; (5) presentación digital y un solo ejemplar empastado (comisión: 7 ejemplares); (6) se agregaron el diplomado, la excelencia, el PETAENG y el examen de técnico superior; (7) se unificó la escala de calificación, que en la comisión tenía tres versiones. ERRORES DE LA COMISIÓN CORREGIDOS: el Art. 73 remitía a los Arts. 42 a 44 (eran el 69 a 71); el Art. 47 remitía al Art. 2 por los requisitos (era el 5); en el trabajo dirigido, el tribunal examinador se formaba con un "tribunal revisor" que esa modalidad no tiene; "Gobierno Corporativo" y "Legislación Tributaria y Aduanera" se cambiaron por los nombres de la malla 2027. Se omitió la cita del "Art. 41 del Reglamento General de Tipos de Modalidad de Graduación del XII Congreso realizado en Oruro": según el diagnóstico, el congreso realizado en Oruro fue el XI (2009), así que el número del congreso o la sede es incorrecto; VERIFICAR el artículo y el congreso.
-ACTUALIZADO (Art. 45, Transición): los egresados del Plan 2013 tienen hasta 3 años desde su egreso para graduarse según la reglamentación de ese plan; luego se rigen por el nuevo reglamento o el PETAENG. Así coincide con la disposición transitoria de la fuente terciaria (punto 16).</t>
+ACTUALIZADO (Art. 45, Transición): los egresados del Plan 2013 tienen hasta 3 años desde su egreso para graduarse según la reglamentación de ese plan; luego se rigen por el nuevo reglamento o el PETAENG. Así coincide con la disposición transitoria de la fuente terciaria (punto 16).
+Actualizado el 14/10/2026 con los documentos pilares: normativa con HCU 139/2013 y 426/2024; reglamentos internos vigentes de 2013 (biblioteca, Internet, incompatibilidad docente, manual de funciones).</t>
         </is>
       </c>
       <c r="J116" s="6" t="n">

</xml_diff>